<commit_message>
[Refactor] TrainData 엑셀 컬럼 active/passive 분리 완료
- TrainData.xlsx: train_skill_data_id 제거, passive_skill_data_id 옆에 active_skill_data_id 컬럼 추가 (sheet1/2/3)
  - TrainRow.cs: passiveSkillDataIds 필드를 base로 끌어올리고 active 컬럼명을 active_skill_data_id로 변경
  - RangeTrainRow.cs / TurretTrainRow.cs: 자체 passiveSkillDataIds 필드 제거 (base 사용)
  - TrainImporter.cs / RangeTrainImporter.cs / TurretTrainImporter.cs: Headers 배열 새 컬럼 순서로 갱신
  - TrainDataReflector.cs: passiveSkillDataIds SetPrivateField 추가
  - TrainData.cs: legacy trainSkillDataIds 필드 및 GetResolvedActiveSkillDataId fallback 제거
</commit_message>
<xml_diff>
--- a/Assets/02_Resources/Data/TrainData.xlsx
+++ b/Assets/02_Resources/Data/TrainData.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="121">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -382,6 +382,9 @@
   </si>
   <si>
     <t xml:space="preserve">50006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">active_skill_data_id</t>
   </si>
 </sst>
 </file>
@@ -800,7 +803,7 @@
   <sheetPr codeName="Sheet1">
     <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="0"/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="3" max="3" width="24.140625" style="1" bestFit="1" customWidth="1"/>
@@ -829,7 +832,10 @@
         <v>6</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>7</v>
+        <v>20</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.55">
@@ -897,34 +903,34 @@
         <v>6</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J1" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K1" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="L1" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M1" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N1" s="0" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="O1" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P1" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q1" s="0" t="s">
-        <v>20</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.55">
@@ -949,28 +955,28 @@
       <c r="G2" s="0" t="s">
         <v>25</v>
       </c>
+      <c r="H2" s="0">
+        <v>5</v>
+      </c>
       <c r="I2" s="0">
         <v>5</v>
       </c>
       <c r="J2" s="0">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="K2" s="0">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="L2" s="0">
-        <v>1</v>
-      </c>
-      <c r="M2" s="0">
         <v>4</v>
       </c>
-      <c r="N2" s="0" t="s">
+      <c r="M2" s="0" t="s">
         <v>26</v>
       </c>
+      <c r="N2" s="0">
+        <v>30</v>
+      </c>
       <c r="O2" s="0">
-        <v>30</v>
-      </c>
-      <c r="P2" s="0">
         <v>0.3</v>
       </c>
     </row>
@@ -996,28 +1002,28 @@
       <c r="G3" s="0" t="s">
         <v>31</v>
       </c>
+      <c r="H3" s="0">
+        <v>5</v>
+      </c>
       <c r="I3" s="0">
         <v>5</v>
       </c>
       <c r="J3" s="0">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K3" s="0">
         <v>1</v>
       </c>
       <c r="L3" s="0">
-        <v>1</v>
-      </c>
-      <c r="M3" s="0">
         <v>0.1</v>
       </c>
-      <c r="N3" s="0" t="s">
+      <c r="M3" s="0" t="s">
         <v>32</v>
       </c>
+      <c r="N3" s="0">
+        <v>30</v>
+      </c>
       <c r="O3" s="0">
-        <v>30</v>
-      </c>
-      <c r="P3" s="0">
         <v>0.3</v>
       </c>
     </row>
@@ -1037,32 +1043,32 @@
       <c r="F4" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="0" t="s">
-        <v>36</v>
+      <c r="H4" s="0">
+        <v>8</v>
       </c>
       <c r="I4" s="0">
         <v>8</v>
       </c>
       <c r="J4" s="0">
-        <v>8</v>
+        <v>500</v>
       </c>
       <c r="K4" s="0">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="L4" s="0">
-        <v>1</v>
-      </c>
-      <c r="M4" s="0">
         <v>4</v>
       </c>
-      <c r="N4" s="0" t="s">
+      <c r="M4" s="0" t="s">
         <v>26</v>
       </c>
+      <c r="N4" s="0">
+        <v>30</v>
+      </c>
       <c r="O4" s="0">
-        <v>30</v>
-      </c>
-      <c r="P4" s="0">
         <v>0.3</v>
+      </c>
+      <c r="Q4" s="0">
+        <v>50008</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.55">
@@ -1081,32 +1087,32 @@
       <c r="F5" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="H5" s="0" t="s">
-        <v>40</v>
+      <c r="H5" s="0">
+        <v>13</v>
       </c>
       <c r="I5" s="0">
         <v>13</v>
       </c>
       <c r="J5" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K5" s="0">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="L5" s="0">
-        <v>1</v>
-      </c>
-      <c r="M5" s="0">
         <v>0.1</v>
       </c>
-      <c r="N5" s="0" t="s">
+      <c r="M5" s="0" t="s">
         <v>32</v>
       </c>
+      <c r="N5" s="0">
+        <v>30</v>
+      </c>
       <c r="O5" s="0">
-        <v>30</v>
-      </c>
-      <c r="P5" s="0">
         <v>0.3</v>
+      </c>
+      <c r="Q5" s="0">
+        <v>50009</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.55">
@@ -1125,35 +1131,35 @@
       <c r="F6" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="H6" s="0" t="s">
-        <v>36</v>
+      <c r="H6" s="0">
+        <v>8</v>
       </c>
       <c r="I6" s="0">
         <v>8</v>
       </c>
       <c r="J6" s="0">
-        <v>8</v>
+        <v>500</v>
       </c>
       <c r="K6" s="0">
-        <v>500</v>
+        <v>1</v>
       </c>
       <c r="L6" s="0">
-        <v>1</v>
-      </c>
-      <c r="M6" s="0">
         <v>4</v>
       </c>
-      <c r="N6" s="0" t="s">
+      <c r="M6" s="0" t="s">
         <v>26</v>
       </c>
+      <c r="N6" s="0">
+        <v>30</v>
+      </c>
       <c r="O6" s="0">
-        <v>30</v>
-      </c>
-      <c r="P6" s="0">
         <v>0.3</v>
       </c>
-      <c r="Q6" s="0" t="s">
+      <c r="P6" s="0" t="s">
         <v>42</v>
+      </c>
+      <c r="Q6" s="0">
+        <v>50008</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.55">
@@ -1172,35 +1178,35 @@
       <c r="F7" s="0" t="s">
         <v>39</v>
       </c>
-      <c r="H7" s="0" t="s">
-        <v>40</v>
+      <c r="H7" s="0">
+        <v>13</v>
       </c>
       <c r="I7" s="0">
         <v>13</v>
       </c>
       <c r="J7" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K7" s="0">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="L7" s="0">
-        <v>1</v>
-      </c>
-      <c r="M7" s="0">
         <v>0.1</v>
       </c>
-      <c r="N7" s="0" t="s">
+      <c r="M7" s="0" t="s">
         <v>32</v>
       </c>
+      <c r="N7" s="0">
+        <v>30</v>
+      </c>
       <c r="O7" s="0">
-        <v>30</v>
-      </c>
-      <c r="P7" s="0">
         <v>0.3</v>
       </c>
-      <c r="Q7" s="0" t="s">
+      <c r="P7" s="0" t="s">
         <v>44</v>
+      </c>
+      <c r="Q7" s="0">
+        <v>50009</v>
       </c>
     </row>
   </sheetData>
@@ -1249,37 +1255,37 @@
         <v>6</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="I1" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J1" s="0" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K1" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="L1" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="M1" s="0" t="s">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="N1" s="0" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O1" s="0" t="s">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="P1" s="0" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q1" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R1" s="0" t="s">
-        <v>20</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.55">
@@ -1304,6 +1310,9 @@
       <c r="G2" s="0" t="s">
         <v>51</v>
       </c>
+      <c r="H2" s="0">
+        <v>10</v>
+      </c>
       <c r="I2" s="0">
         <v>10</v>
       </c>
@@ -1311,24 +1320,21 @@
         <v>10</v>
       </c>
       <c r="K2" s="0">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L2" s="0">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="M2" s="0">
-        <v>0.3</v>
-      </c>
-      <c r="N2" s="0">
-        <v>1</v>
-      </c>
-      <c r="O2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="N2" s="0" t="s">
         <v>52</v>
       </c>
+      <c r="O2" s="0">
+        <v>30</v>
+      </c>
       <c r="P2" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q2" s="0">
         <v>0.3</v>
       </c>
     </row>
@@ -1354,31 +1360,31 @@
       <c r="G3" s="0" t="s">
         <v>57</v>
       </c>
+      <c r="H3" s="0">
+        <v>8</v>
+      </c>
       <c r="I3" s="0">
         <v>8</v>
       </c>
       <c r="J3" s="0">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K3" s="0">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L3" s="0">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="M3" s="0">
-        <v>0.15</v>
-      </c>
-      <c r="N3" s="0">
-        <v>1</v>
-      </c>
-      <c r="O3" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="N3" s="0" t="s">
         <v>58</v>
       </c>
+      <c r="O3" s="0">
+        <v>30</v>
+      </c>
       <c r="P3" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q3" s="0">
         <v>0.3</v>
       </c>
     </row>
@@ -1404,31 +1410,31 @@
       <c r="G4" s="0" t="s">
         <v>63</v>
       </c>
+      <c r="H4" s="0">
+        <v>10</v>
+      </c>
       <c r="I4" s="0">
         <v>10</v>
       </c>
       <c r="J4" s="0">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="K4" s="0">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L4" s="0">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="M4" s="0">
-        <v>1.25</v>
-      </c>
-      <c r="N4" s="0">
-        <v>1</v>
-      </c>
-      <c r="O4" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="N4" s="0" t="s">
         <v>64</v>
       </c>
+      <c r="O4" s="0">
+        <v>30</v>
+      </c>
       <c r="P4" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q4" s="0">
         <v>0.3</v>
       </c>
     </row>
@@ -1454,31 +1460,31 @@
       <c r="G5" s="0" t="s">
         <v>69</v>
       </c>
+      <c r="H5" s="0">
+        <v>30</v>
+      </c>
       <c r="I5" s="0">
         <v>30</v>
       </c>
       <c r="J5" s="0">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="K5" s="0">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="L5" s="0">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="M5" s="0">
-        <v>2.5</v>
-      </c>
-      <c r="N5" s="0">
-        <v>1</v>
-      </c>
-      <c r="O5" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="N5" s="0" t="s">
         <v>70</v>
       </c>
+      <c r="O5" s="0">
+        <v>30</v>
+      </c>
       <c r="P5" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q5" s="0">
         <v>0.3</v>
       </c>
     </row>
@@ -1504,31 +1510,31 @@
       <c r="G6" s="0" t="s">
         <v>75</v>
       </c>
+      <c r="H6" s="0">
+        <v>20</v>
+      </c>
       <c r="I6" s="0">
         <v>20</v>
       </c>
       <c r="J6" s="0">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K6" s="0">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="L6" s="0">
+        <v>1</v>
+      </c>
+      <c r="M6" s="0">
         <v>3</v>
       </c>
-      <c r="M6" s="0">
-        <v>1</v>
-      </c>
-      <c r="N6" s="0">
-        <v>3</v>
-      </c>
-      <c r="O6" s="0" t="s">
+      <c r="N6" s="0" t="s">
         <v>76</v>
       </c>
+      <c r="O6" s="0">
+        <v>30</v>
+      </c>
       <c r="P6" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q6" s="0">
         <v>0.3</v>
       </c>
     </row>
@@ -1554,31 +1560,31 @@
       <c r="G7" s="0" t="s">
         <v>81</v>
       </c>
+      <c r="H7" s="0">
+        <v>3</v>
+      </c>
       <c r="I7" s="0">
         <v>3</v>
       </c>
       <c r="J7" s="0">
+        <v>50</v>
+      </c>
+      <c r="K7" s="0">
+        <v>1</v>
+      </c>
+      <c r="L7" s="0">
         <v>3</v>
       </c>
-      <c r="K7" s="0">
-        <v>50</v>
-      </c>
-      <c r="L7" s="0">
-        <v>1</v>
-      </c>
       <c r="M7" s="0">
-        <v>3</v>
-      </c>
-      <c r="N7" s="0">
-        <v>1</v>
-      </c>
-      <c r="O7" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="N7" s="0" t="s">
         <v>82</v>
       </c>
+      <c r="O7" s="0">
+        <v>30</v>
+      </c>
       <c r="P7" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q7" s="0">
         <v>0.3</v>
       </c>
     </row>
@@ -1604,14 +1610,17 @@
       <c r="G8" s="0" t="s">
         <v>87</v>
       </c>
+      <c r="H8" s="0">
+        <v>30</v>
+      </c>
       <c r="I8" s="0">
         <v>30</v>
       </c>
       <c r="J8" s="0">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="K8" s="0">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="L8" s="0">
         <v>1</v>
@@ -1619,16 +1628,13 @@
       <c r="M8" s="0">
         <v>1</v>
       </c>
-      <c r="N8" s="0">
-        <v>1</v>
-      </c>
-      <c r="O8" s="0" t="s">
+      <c r="N8" s="0" t="s">
         <v>88</v>
       </c>
+      <c r="O8" s="0">
+        <v>30</v>
+      </c>
       <c r="P8" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q8" s="0">
         <v>0.3</v>
       </c>
     </row>
@@ -1652,38 +1658,38 @@
       <c r="G9" s="0" t="s">
         <v>51</v>
       </c>
-      <c r="H9" s="0" t="s">
-        <v>117</v>
+      <c r="H9" s="0">
+        <v>10</v>
       </c>
       <c r="I9" s="0">
         <v>10</v>
       </c>
       <c r="J9" s="0">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="K9" s="0">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="L9" s="0">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="M9" s="0">
-        <v>0.1</v>
-      </c>
-      <c r="N9" s="0">
-        <v>0</v>
-      </c>
-      <c r="O9" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N9" s="0" t="s">
         <v>52</v>
       </c>
+      <c r="O9" s="0">
+        <v>30</v>
+      </c>
       <c r="P9" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q9" s="0">
         <v>0.3</v>
       </c>
-      <c r="R9" s="0" t="s">
+      <c r="Q9" s="0" t="s">
         <v>103</v>
+      </c>
+      <c r="R9" s="0">
+        <v>50001</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.55">
@@ -1706,34 +1712,34 @@
       <c r="G10" s="0" t="s">
         <v>57</v>
       </c>
+      <c r="H10" s="0">
+        <v>10</v>
+      </c>
       <c r="I10" s="0">
         <v>10</v>
       </c>
       <c r="J10" s="0">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="K10" s="0">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L10" s="0">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="M10" s="0">
-        <v>0.1</v>
-      </c>
-      <c r="N10" s="0">
-        <v>0</v>
-      </c>
-      <c r="O10" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N10" s="0" t="s">
         <v>58</v>
       </c>
+      <c r="O10" s="0">
+        <v>30</v>
+      </c>
       <c r="P10" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q10" s="0">
         <v>0.3</v>
       </c>
-      <c r="R10" s="0" t="s">
+      <c r="Q10" s="0" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1757,34 +1763,34 @@
       <c r="G11" s="0" t="s">
         <v>63</v>
       </c>
+      <c r="H11" s="0">
+        <v>10</v>
+      </c>
       <c r="I11" s="0">
         <v>10</v>
       </c>
       <c r="J11" s="0">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="K11" s="0">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="L11" s="0">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="M11" s="0">
-        <v>0.5</v>
-      </c>
-      <c r="N11" s="0">
-        <v>0</v>
-      </c>
-      <c r="O11" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N11" s="0" t="s">
         <v>64</v>
       </c>
+      <c r="O11" s="0">
+        <v>30</v>
+      </c>
       <c r="P11" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q11" s="0">
         <v>0.3</v>
       </c>
-      <c r="R11" s="0" t="s">
+      <c r="Q11" s="0" t="s">
         <v>105</v>
       </c>
     </row>
@@ -1808,34 +1814,34 @@
       <c r="G12" s="0" t="s">
         <v>69</v>
       </c>
+      <c r="H12" s="0">
+        <v>30</v>
+      </c>
       <c r="I12" s="0">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="J12" s="0">
-        <v>10</v>
+        <v>300</v>
       </c>
       <c r="K12" s="0">
-        <v>300</v>
+        <v>1</v>
       </c>
       <c r="L12" s="0">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M12" s="0">
-        <v>3</v>
-      </c>
-      <c r="N12" s="0">
-        <v>0</v>
-      </c>
-      <c r="O12" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N12" s="0" t="s">
         <v>70</v>
       </c>
+      <c r="O12" s="0">
+        <v>30</v>
+      </c>
       <c r="P12" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q12" s="0">
         <v>0.3</v>
       </c>
-      <c r="R12" s="0" t="s">
+      <c r="Q12" s="0" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1859,38 +1865,38 @@
       <c r="G13" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="H13" s="0" t="s">
-        <v>118</v>
+      <c r="H13" s="0">
+        <v>10</v>
       </c>
       <c r="I13" s="0">
         <v>10</v>
       </c>
       <c r="J13" s="0">
-        <v>10</v>
+        <v>400</v>
       </c>
       <c r="K13" s="0">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="L13" s="0">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M13" s="0">
-        <v>5</v>
-      </c>
-      <c r="N13" s="0">
-        <v>0</v>
-      </c>
-      <c r="O13" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N13" s="0" t="s">
         <v>76</v>
       </c>
+      <c r="O13" s="0">
+        <v>30</v>
+      </c>
       <c r="P13" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q13" s="0">
         <v>0.3</v>
       </c>
-      <c r="R13" s="0" t="s">
+      <c r="Q13" s="0" t="s">
         <v>107</v>
+      </c>
+      <c r="R13" s="0">
+        <v>50005</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.55">
@@ -1913,38 +1919,38 @@
       <c r="G14" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="H14" s="0" t="s">
-        <v>119</v>
+      <c r="H14" s="0">
+        <v>10</v>
       </c>
       <c r="I14" s="0">
         <v>10</v>
       </c>
       <c r="J14" s="0">
-        <v>10</v>
+        <v>400</v>
       </c>
       <c r="K14" s="0">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="L14" s="0">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M14" s="0">
-        <v>3</v>
-      </c>
-      <c r="N14" s="0">
-        <v>0</v>
-      </c>
-      <c r="O14" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N14" s="0" t="s">
         <v>82</v>
       </c>
+      <c r="O14" s="0">
+        <v>30</v>
+      </c>
       <c r="P14" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q14" s="0">
         <v>0.3</v>
       </c>
-      <c r="R14" s="0" t="s">
+      <c r="Q14" s="0" t="s">
         <v>108</v>
+      </c>
+      <c r="R14" s="0">
+        <v>50006</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.55">
@@ -1967,34 +1973,34 @@
       <c r="G15" s="0" t="s">
         <v>87</v>
       </c>
+      <c r="H15" s="0">
+        <v>10</v>
+      </c>
       <c r="I15" s="0">
         <v>10</v>
       </c>
       <c r="J15" s="0">
-        <v>10</v>
+        <v>600</v>
       </c>
       <c r="K15" s="0">
-        <v>600</v>
+        <v>1</v>
       </c>
       <c r="L15" s="0">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="M15" s="0">
-        <v>1.5</v>
-      </c>
-      <c r="N15" s="0">
-        <v>0</v>
-      </c>
-      <c r="O15" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="N15" s="0" t="s">
         <v>88</v>
       </c>
+      <c r="O15" s="0">
+        <v>30</v>
+      </c>
       <c r="P15" s="0">
-        <v>30</v>
-      </c>
-      <c r="Q15" s="0">
         <v>0.3</v>
       </c>
-      <c r="R15" s="0" t="s">
+      <c r="Q15" s="0" t="s">
         <v>109</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[Fix] turret 시트 max_hp xlsx/DB 불일치 정리
- TrainData.xlsx: turret max_hp 옛값 250 → DB 일치 150으로 수정 (30001~31007, 14행)
</commit_message>
<xml_diff>
--- a/Assets/02_Resources/Data/TrainData.xlsx
+++ b/Assets/02_Resources/Data/TrainData.xlsx
@@ -1319,7 +1319,7 @@
         <v>78</v>
       </c>
       <c r="D2" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E2" s="3">
         <v>0</v>
@@ -1369,7 +1369,7 @@
         <v>47</v>
       </c>
       <c r="D3" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E3" s="3">
         <v>0</v>
@@ -1419,7 +1419,7 @@
         <v>66</v>
       </c>
       <c r="D4" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E4" s="3">
         <v>0</v>
@@ -1469,7 +1469,7 @@
         <v>30</v>
       </c>
       <c r="D5" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E5" s="3">
         <v>0</v>
@@ -1519,7 +1519,7 @@
         <v>61</v>
       </c>
       <c r="D6" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E6" s="3">
         <v>0</v>
@@ -1569,7 +1569,7 @@
         <v>59</v>
       </c>
       <c r="D7" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E7" s="3">
         <v>0</v>
@@ -1619,7 +1619,7 @@
         <v>42</v>
       </c>
       <c r="D8" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E8" s="3">
         <v>0</v>
@@ -1667,7 +1667,7 @@
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E9" s="3">
         <v>0</v>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E10" s="3">
         <v>0</v>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E11" s="3">
         <v>0</v>
@@ -1824,7 +1824,7 @@
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E12" s="3">
         <v>0</v>
@@ -1875,7 +1875,7 @@
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E13" s="3">
         <v>0</v>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E14" s="3">
         <v>0</v>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="E15" s="3">
         <v>0</v>

</xml_diff>